<commit_message>
R05 (em andamento): relatório (rascunho), HISTORICO, README e LEIAME do quadro (sobra da E4 e EOB implícito das latentes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/resultados/rodada05/quadro_subsetores_v04.xlsx
+++ b/resultados/rodada05/quadro_subsetores_v04.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -469,19 +469,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abas: v03_x_v04 (comparativo por subsetor), passos_v03_v04 (efeito de D17 e D18), d18_latentes (τ_RS, p_k, coeficiente de TUST e multiplicadores das latentes sem e com a D18), tust_latentes_versoes, realocacao_E4 (valores movidos na variante _E4), insumos_nao_energeticos (T12), tust_geracao, pisos_vbp, reequilibrio_RAS, reequilibrio_insumos, variantes_resumo e variantes_subsetores, gas_por_comprador e gas_por_grupo, checagens de todas as versões, niveis_emissoes.</t>
+          <t>Abas: v03_x_v04 (comparativo por subsetor), passos_v03_v04 (efeito de D17 e D18), d18_latentes (τ_RS, p_k, coeficiente de TUST e multiplicadores das latentes sem e com a D18; EOB/VBP implícito das latentes), d18_eob_implicito_versoes (o mesmo nas 9 versões; o PET-RS latente fica abaixo de η), tust_latentes_versoes, realocacao_E4 (valores movidos na variante _E4), insumos_nao_energeticos (T12), tust_geracao, pisos_vbp, reequilibrio_RAS, reequilibrio_insumos, variantes_resumo e variantes_subsetores, gas_por_comprador e gas_por_grupo, checagens de todas as versões, niveis_emissoes.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GWh (D8): Brasil pelo BEN 2020 (Tabela 5.4), RS pelo ONS, RB = Brasil − RS.</t>
+          <t>realocacao_E4: sai de DIS e GAS só a parte de resíduo da E1, na proporção do resíduo de cada um (= do VBP); o SF₆, nível identificado na E1, fica. O que sobra em DIS + GAS = resíduo não movido + SF₆ do DIS; é esse total que corresponde à sobra de referência das instruções (Seção 3.2).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>GWh (D8): Brasil pelo BEN 2020 (Tabela 5.4), RS pelo ONS, RB = Brasil − RS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Gerado por scripts/rodada05_mip.py.</t>
         </is>

</xml_diff>